<commit_message>
Actualización: agregado benchmark, encuestas, entrevistas y otros documentos. Eliminado CSV antiguo.
</commit_message>
<xml_diff>
--- a/01-planificacion/Investigar cómo los usuarios actualmente buscan planes de nutrición_ejercicio..xlsx
+++ b/01-planificacion/Investigar cómo los usuarios actualmente buscan planes de nutrición_ejercicio..xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Estudio\Iberoamericana\Analisis y diseño de sistemas\Repositorio\01-planificacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E5168FD-B314-4656-A98D-C8DDF3E091E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D30DBE9-4F28-433D-AE7B-D36AC4523286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{08D700EA-4E28-4F26-AADC-108F0AC1958A}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t>Fuente</t>
   </si>
@@ -113,13 +113,108 @@
   </si>
   <si>
     <t>Cómo buscan actualmente planes de nutrición y ejercicio</t>
+  </si>
+  <si>
+    <t>Categoría</t>
+  </si>
+  <si>
+    <t>Problema identificado</t>
+  </si>
+  <si>
+    <t>Fuente/Ejemplo</t>
+  </si>
+  <si>
+    <t>Nutrición</t>
+  </si>
+  <si>
+    <t>Dietas genéricas sin personalización real, que no consideran gustos, alergias o restricciones.</t>
+  </si>
+  <si>
+    <t>Reportes de usuarios en apps como MyFitnessPal.</t>
+  </si>
+  <si>
+    <t>Dificultad para dar seguimiento real a lo que se come (usuarios olvidan registrar).</t>
+  </si>
+  <si>
+    <t>Blog de DietDoctor, 2023.</t>
+  </si>
+  <si>
+    <t>Ejercicio</t>
+  </si>
+  <si>
+    <t>Sedentarismo en trabajadores remotos que no logran organizar pausas activas.</t>
+  </si>
+  <si>
+    <t>Encuestas OMS sobre actividad física.</t>
+  </si>
+  <si>
+    <t>Falta de motivación para mantener rutinas más de 2-3 semanas.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Estudio de </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Journal of Behavioral Medicine</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Tecnología</t>
+  </si>
+  <si>
+    <t>Tener que usar varias apps separadas (una de dieta, otra de ejercicio, otra de recordatorios).</t>
+  </si>
+  <si>
+    <t>Opiniones en foros de Reddit sobre apps fitness.</t>
+  </si>
+  <si>
+    <t>Interfaces poco intuitivas, abandono por complejidad de uso.</t>
+  </si>
+  <si>
+    <t>Análisis UX en Medium, 2022.</t>
+  </si>
+  <si>
+    <t>Usuarios</t>
+  </si>
+  <si>
+    <t>Frustración al no ver resultados rápidos.</t>
+  </si>
+  <si>
+    <t>Estudio motivacional de apps de salud digital.</t>
+  </si>
+  <si>
+    <t>Falta de acompañamiento humano o de IA que dé feedback oportuno.</t>
+  </si>
+  <si>
+    <t>Opiniones en App Store/Google Play.</t>
+  </si>
+  <si>
+    <t>Recolectar ejemplos de problemas reales</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,6 +248,14 @@
       <b/>
       <sz val="16"/>
       <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -342,6 +445,60 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>350226</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>28024</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1919654" cy="578001"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2" descr="Imagen generada">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB5DA454-04F7-45BF-9D55-68E06BECBF15}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect t="25202" b="29725"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="1112226" y="4563389"/>
+          <a:ext cx="1919654" cy="578001"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -823,7 +980,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F24226D7-5B8D-4B9E-92D7-85DD646C8359}">
-  <dimension ref="B2:E8"/>
+  <dimension ref="B2:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="40.5703125" customWidth="1"/>
@@ -853,7 +1010,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
@@ -867,7 +1024,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
@@ -923,9 +1080,115 @@
         <v>23</v>
       </c>
     </row>
+    <row r="11" spans="2:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="5"/>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C11:D11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>